<commit_message>
Nettoyage BAAC (Phase 2) + migration suivi projet vers OneDrive + renommage catalogue/
</commit_message>
<xml_diff>
--- a/Catalogue/Catalogue_final.xlsx
+++ b/Catalogue/Catalogue_final.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\PROJET\PHASES\0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\mobilite-securite-routiere\Catalogue\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -231,9 +231,6 @@
     <t>Problèmes de qualité anticipés</t>
   </si>
   <si>
-    <t>Base nationale à filtrer sur Paris (dep=75) ; vérifier valeurs manquantes sur lat/long ; codes de gravité à retraiter en cible binaire ; encodage des accents à corriger (caractères mal affichés observés, ex. 'Ã©') ; vérifier la clé de jointure entre le fichier véhicules immatriculés et les 4 fichiers BAAC standards</t>
-  </si>
-  <si>
     <t>Colonne 'dessin' lourde et redondante avec le référentiel géo, à exclure du chargement ; etat_trafic/etat_barre codés en entiers ici (contrairement à l'API '13 mois glissants' qui les donne en texte) — prévoir une table de correspondance ; valeurs q/k parfois absentes selon les tronçons</t>
   </si>
   <si>
@@ -370,6 +367,9 @@
   </si>
   <si>
     <t>Référentiel géographique</t>
+  </si>
+  <si>
+    <t>Base nationale à filtrer sur Paris (dep=75) ; vérifier valeurs manquantes sur lat/long ; codes de gravité à retraiter en cible binaire ; encodage des accents à corriger (caractères mal affichés observés, ex. 'Ã©') ; vérifier la clé de jointure entre le fichier véhicules immatriculés et les 4 fichiers BAAC standards / Fichier exclu du pipeline final — clé Id_accident incompatible avec Num_Acc, aucune table de correspondance disponible</t>
   </si>
 </sst>
 </file>
@@ -494,10 +494,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -772,15 +772,15 @@
     <col min="7" max="16384" width="8.6328125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="8" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
+    <row r="1" spans="1:6" s="7" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
     </row>
     <row r="2" spans="1:6" ht="39" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
@@ -793,7 +793,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>3</v>
@@ -1022,84 +1022,84 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="119.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ht="154" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>67</v>
       </c>
       <c r="B14" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="53" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="46" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="C17" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1121,7 +1121,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
@@ -1129,37 +1129,37 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
@@ -1167,17 +1167,17 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
@@ -1185,22 +1185,22 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
@@ -1208,32 +1208,32 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
@@ -1241,12 +1241,12 @@
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>